<commit_message>
v1.0 + Auth + QR Platform working end to end
</commit_message>
<xml_diff>
--- a/bulk_qr_output/bulk_qr_status.xlsx
+++ b/bulk_qr_output/bulk_qr_status.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,12 +455,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://futuretechsolution.in</t>
+          <t>www:futuretechsolution.in</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Failed</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://openai.com</t>
+          <t>openai.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Failed</t>
         </is>
       </c>
     </row>

</xml_diff>